<commit_message>
Added template therion project to test the processing of transcribed W.Stanton log book data
SVN-Revision: r5
SVN-URL: https://www.cave-registry.org.uk/svn/WookeyCatchment/Swildons
</commit_message>
<xml_diff>
--- a/WISLogbookTranscription/WStantonSurveyBook1p49-58.xlsx
+++ b/WISLogbookTranscription/WStantonSurveyBook1p49-58.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
     <sheet name="Interpreted Data" sheetId="2" r:id="rId2"/>
     <sheet name="Survex Formatted" sheetId="3" r:id="rId3"/>
+    <sheet name="Therion Formatted" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="145621"/>
 </workbook>
@@ -206,7 +207,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -252,15 +253,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -268,66 +266,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -676,10 +624,10 @@
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="2"/>
+      <c r="F2" s="8"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -737,40 +685,40 @@
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>20</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="6">
         <v>4</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="6">
         <v>103</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="6">
         <v>283</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="6">
         <v>21</v>
       </c>
-      <c r="K4" s="7">
+      <c r="K4" s="6">
         <v>8.5</v>
       </c>
-      <c r="M4" s="7">
+      <c r="M4" s="6">
         <v>20.8</v>
       </c>
-      <c r="N4" s="7">
+      <c r="N4" s="6">
         <v>3.1</v>
       </c>
       <c r="P4" t="s">
@@ -781,43 +729,43 @@
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <v>6</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <v>3.5</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="6">
         <v>3</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="6">
         <v>6</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="I5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="6">
         <v>27</v>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="6">
         <v>-9.5</v>
       </c>
       <c r="M5">
         <v>26.7</v>
       </c>
-      <c r="N5" s="7">
+      <c r="N5" s="6">
         <v>-4.5</v>
       </c>
-      <c r="O5" s="7">
+      <c r="O5" s="6">
         <v>3.1</v>
       </c>
     </row>
@@ -825,43 +773,43 @@
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>7</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="6">
         <v>4</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="6">
         <v>2</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="6">
         <v>83</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="6">
         <v>263</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="6">
         <v>37</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="M6" s="7">
+      <c r="M6" s="6">
         <v>37</v>
       </c>
-      <c r="N6" s="7">
+      <c r="N6" s="6">
         <v>1.5</v>
       </c>
-      <c r="O6" s="7">
+      <c r="O6" s="6">
         <v>-1.4</v>
       </c>
     </row>
@@ -869,43 +817,43 @@
       <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <v>25</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <v>2</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="6">
         <v>10</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="6">
         <v>16.2</v>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="6">
         <v>4.3</v>
       </c>
       <c r="M7">
         <v>16.100000000000001</v>
       </c>
-      <c r="N7" s="7">
+      <c r="N7" s="6">
         <v>1.3</v>
       </c>
-      <c r="O7" s="7">
+      <c r="O7" s="6">
         <v>0.1</v>
       </c>
     </row>
@@ -913,43 +861,43 @@
       <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="6">
         <v>25</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <v>4.5</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="6">
         <v>6</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="6">
         <v>78</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="6">
         <v>258</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="6">
         <v>47</v>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="6">
         <v>-5.3</v>
       </c>
-      <c r="M8" s="7">
+      <c r="M8" s="6">
         <v>46.8</v>
       </c>
-      <c r="N8" s="7">
+      <c r="N8" s="6">
         <v>-4.5</v>
       </c>
-      <c r="O8" s="7">
+      <c r="O8" s="6">
         <v>1.4</v>
       </c>
     </row>
@@ -957,43 +905,43 @@
       <c r="A9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="6">
         <v>4</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="6">
         <v>2</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="6">
         <v>0.5</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="6">
         <v>292</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="6">
         <v>292</v>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="6">
         <v>48</v>
       </c>
-      <c r="K9" s="7" t="s">
+      <c r="K9" s="6" t="s">
         <v>53</v>
       </c>
       <c r="M9">
         <v>48</v>
       </c>
-      <c r="N9" s="7">
+      <c r="N9" s="6">
         <v>-2.5</v>
       </c>
-      <c r="O9" s="7">
+      <c r="O9" s="6">
         <v>-3.1</v>
       </c>
     </row>
@@ -1001,43 +949,43 @@
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="6">
         <v>2.5</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="6">
         <v>0.5</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="6">
         <v>3.5</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="6">
         <v>7</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="6">
         <v>159</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="6">
         <v>339</v>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="6">
         <v>36</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="K10" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="M10" s="7">
+      <c r="M10" s="6">
         <v>36</v>
       </c>
       <c r="N10" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="7">
+      <c r="O10" s="6">
         <v>-5.6</v>
       </c>
     </row>
@@ -1045,43 +993,43 @@
       <c r="A11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="6">
         <v>15</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="6">
         <v>1</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="6">
         <v>10</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="6">
         <v>3</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="6">
         <v>247</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="6">
         <v>247</v>
       </c>
-      <c r="J11" s="7">
+      <c r="J11" s="6">
         <v>31</v>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="6">
         <v>-2.2999999999999998</v>
       </c>
-      <c r="M11" s="7">
+      <c r="M11" s="6">
         <v>31</v>
       </c>
-      <c r="N11" s="7">
+      <c r="N11" s="6">
         <v>-1.3</v>
       </c>
-      <c r="O11" s="7">
+      <c r="O11" s="6">
         <v>-5.6</v>
       </c>
     </row>
@@ -1089,43 +1037,43 @@
       <c r="A12" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="6">
         <v>15</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="6">
         <v>1</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="6">
         <v>8</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="6">
         <v>2</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="6">
         <v>95</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="6">
         <v>275</v>
       </c>
-      <c r="J12" s="7">
+      <c r="J12" s="6">
         <v>26</v>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="6">
         <v>2</v>
       </c>
-      <c r="M12" s="7">
+      <c r="M12" s="6">
         <v>26</v>
       </c>
-      <c r="N12" s="7">
+      <c r="N12" s="6">
         <v>0.9</v>
       </c>
-      <c r="O12" s="7">
+      <c r="O12" s="6">
         <v>-6.9</v>
       </c>
     </row>
@@ -1133,43 +1081,43 @@
       <c r="A13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="6">
         <v>8</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="6">
         <v>3</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="6">
         <v>1</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="6">
         <v>2</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="6">
         <v>320</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="6">
         <v>320</v>
       </c>
-      <c r="J13" s="7">
+      <c r="J13" s="6">
         <v>26.5</v>
       </c>
-      <c r="K13" s="7">
+      <c r="K13" s="6">
         <v>1</v>
       </c>
-      <c r="M13" s="7">
+      <c r="M13" s="6">
         <v>26.5</v>
       </c>
-      <c r="N13" s="7">
+      <c r="N13" s="6">
         <v>0.5</v>
       </c>
-      <c r="O13" s="7">
+      <c r="O13" s="6">
         <v>-6</v>
       </c>
     </row>
@@ -1177,43 +1125,43 @@
       <c r="A14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="6">
         <v>25</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="6">
         <v>4.5</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14" s="6">
         <v>4</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="6">
         <v>193</v>
       </c>
-      <c r="I14" s="7">
+      <c r="I14" s="6">
         <v>13</v>
       </c>
-      <c r="J14" s="7">
+      <c r="J14" s="6">
         <v>17.5</v>
       </c>
-      <c r="K14" s="7">
+      <c r="K14" s="6">
         <v>-9</v>
       </c>
-      <c r="M14" s="7">
+      <c r="M14" s="6">
         <v>17.3</v>
       </c>
-      <c r="N14" s="7">
+      <c r="N14" s="6">
         <v>-2.7</v>
       </c>
-      <c r="O14" s="7">
+      <c r="O14" s="6">
         <v>-5.5</v>
       </c>
     </row>
@@ -1221,43 +1169,43 @@
       <c r="A15" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="6">
         <v>20</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="6">
         <v>3</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="6">
         <v>2</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="6">
         <v>2</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="6">
         <v>299</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="6">
         <v>299</v>
       </c>
-      <c r="J15" s="7">
+      <c r="J15" s="6">
         <v>33</v>
       </c>
-      <c r="K15" s="7">
+      <c r="K15" s="6">
         <v>-3</v>
       </c>
-      <c r="M15" s="7">
+      <c r="M15" s="6">
         <v>33</v>
       </c>
-      <c r="N15" s="7">
+      <c r="N15" s="6">
         <v>-1.7</v>
       </c>
-      <c r="O15" s="7">
+      <c r="O15" s="6">
         <v>-8.1999999999999993</v>
       </c>
     </row>
@@ -1265,43 +1213,43 @@
       <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="6">
         <v>15</v>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="6">
         <v>7</v>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="6">
         <v>4</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="6">
         <v>142</v>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="6">
         <v>322</v>
       </c>
-      <c r="J16" s="7">
+      <c r="J16" s="6">
         <v>43</v>
       </c>
-      <c r="K16" s="7">
+      <c r="K16" s="6">
         <v>-7.3</v>
       </c>
-      <c r="M16" s="7">
+      <c r="M16" s="6">
         <v>42.7</v>
       </c>
-      <c r="N16" s="7">
+      <c r="N16" s="6">
         <v>-5.6</v>
       </c>
-      <c r="O16" s="7">
+      <c r="O16" s="6">
         <v>-9.9</v>
       </c>
     </row>
@@ -1309,43 +1257,43 @@
       <c r="A17" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="6">
         <v>25</v>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="6">
         <v>3</v>
       </c>
-      <c r="E17" s="7">
+      <c r="E17" s="6">
         <v>2</v>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="6">
         <v>1</v>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="6">
         <v>281</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="H17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="6">
         <v>281</v>
       </c>
-      <c r="J17" s="7">
+      <c r="J17" s="6">
         <v>15.5</v>
       </c>
-      <c r="K17" s="7">
+      <c r="K17" s="6">
         <v>-2</v>
       </c>
-      <c r="M17" s="7">
+      <c r="M17" s="6">
         <v>15.5</v>
       </c>
-      <c r="N17" s="7">
+      <c r="N17" s="6">
         <v>-0.5</v>
       </c>
-      <c r="O17" s="7">
+      <c r="O17" s="6">
         <v>-15.5</v>
       </c>
     </row>
@@ -1353,43 +1301,43 @@
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="6">
         <v>40</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="6">
         <v>4.5</v>
       </c>
-      <c r="E18" s="7">
+      <c r="E18" s="6">
         <v>2</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="6">
         <v>2</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G18" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="6">
         <v>127</v>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="6">
         <v>307</v>
       </c>
-      <c r="J18" s="7">
+      <c r="J18" s="6">
         <v>56</v>
       </c>
-      <c r="K18" s="7">
+      <c r="K18" s="6">
         <v>-5</v>
       </c>
-      <c r="M18" s="7">
+      <c r="M18" s="6">
         <v>55.8</v>
       </c>
-      <c r="N18" s="7">
+      <c r="N18" s="6">
         <v>-4.9000000000000004</v>
       </c>
-      <c r="O18" s="7">
+      <c r="O18" s="6">
         <v>-16</v>
       </c>
     </row>
@@ -1397,43 +1345,43 @@
       <c r="A19" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="6">
         <v>40</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="6">
         <v>3</v>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="6">
         <v>2</v>
       </c>
-      <c r="F19" s="7">
+      <c r="F19" s="6">
         <v>3</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="6">
         <v>283</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="H19" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="6">
         <v>283</v>
       </c>
-      <c r="J19" s="7">
+      <c r="J19" s="6">
         <v>15.8</v>
       </c>
-      <c r="K19" s="7">
+      <c r="K19" s="6">
         <v>-0.15</v>
       </c>
-      <c r="M19" s="7">
+      <c r="M19" s="6">
         <v>15.8</v>
       </c>
-      <c r="N19" s="7">
+      <c r="N19" s="6">
         <v>-0.1</v>
       </c>
-      <c r="O19" s="7">
+      <c r="O19" s="6">
         <v>-20.9</v>
       </c>
     </row>
@@ -1441,43 +1389,43 @@
       <c r="A20" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="6">
         <v>40</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="6">
         <v>4</v>
       </c>
-      <c r="E20" s="7">
+      <c r="E20" s="6">
         <v>4</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="G20" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="6">
         <v>37</v>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="6">
         <v>217</v>
       </c>
-      <c r="J20" s="7">
+      <c r="J20" s="6">
         <v>15.3</v>
       </c>
-      <c r="K20" s="7" t="s">
+      <c r="K20" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="M20" s="7">
+      <c r="M20" s="6">
         <v>15.3</v>
       </c>
-      <c r="N20" s="7">
+      <c r="N20" s="6">
         <v>-4</v>
       </c>
-      <c r="O20" s="7">
+      <c r="O20" s="6">
         <v>-21</v>
       </c>
     </row>
@@ -1485,43 +1433,43 @@
       <c r="A21" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="6">
         <v>40</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="6">
         <v>4</v>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="6">
         <v>310</v>
       </c>
-      <c r="H21" s="7" t="s">
+      <c r="H21" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="6">
         <v>310</v>
       </c>
-      <c r="J21" s="7">
+      <c r="J21" s="6">
         <v>39.5</v>
       </c>
-      <c r="K21" s="7" t="s">
+      <c r="K21" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="M21" s="7">
+      <c r="M21" s="6">
         <v>39.5</v>
       </c>
-      <c r="N21" s="7">
+      <c r="N21" s="6">
         <v>4</v>
       </c>
-      <c r="O21" s="7">
+      <c r="O21" s="6">
         <v>-25</v>
       </c>
     </row>
@@ -1529,43 +1477,43 @@
       <c r="A22" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="7">
+      <c r="C22" s="6">
         <v>12</v>
       </c>
-      <c r="D22" s="7">
+      <c r="D22" s="6">
         <v>4.5</v>
       </c>
-      <c r="E22" s="7">
+      <c r="E22" s="6">
         <v>8</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22" s="6">
         <v>58</v>
       </c>
-      <c r="I22" s="7">
+      <c r="I22" s="6">
         <v>238</v>
       </c>
-      <c r="J22" s="7">
+      <c r="J22" s="6">
         <v>39.6</v>
       </c>
-      <c r="K22" s="7">
+      <c r="K22" s="6">
         <v>-2.7</v>
       </c>
-      <c r="M22" s="7">
+      <c r="M22" s="6">
         <v>39.6</v>
       </c>
-      <c r="N22" s="7">
+      <c r="N22" s="6">
         <v>-1.9</v>
       </c>
-      <c r="O22" s="7">
+      <c r="O22" s="6">
         <v>-21</v>
       </c>
     </row>
@@ -1573,43 +1521,43 @@
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="6">
         <v>2</v>
       </c>
-      <c r="D23" s="7">
+      <c r="D23" s="6">
         <v>2.5</v>
       </c>
-      <c r="E23" s="7">
+      <c r="E23" s="6">
         <v>15</v>
       </c>
-      <c r="F23" s="7">
+      <c r="F23" s="6">
         <v>6</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="6">
         <v>148</v>
       </c>
-      <c r="H23" s="7" t="s">
+      <c r="H23" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I23" s="7">
+      <c r="I23" s="6">
         <v>148</v>
       </c>
-      <c r="J23" s="7">
+      <c r="J23" s="6">
         <v>49</v>
       </c>
-      <c r="K23" s="7" t="s">
+      <c r="K23" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="M23" s="7">
+      <c r="M23" s="6">
         <v>49</v>
       </c>
-      <c r="N23" s="7">
+      <c r="N23" s="6">
         <v>-1.7</v>
       </c>
-      <c r="O23" s="7">
+      <c r="O23" s="6">
         <v>-22.9</v>
       </c>
     </row>
@@ -1617,31 +1565,31 @@
       <c r="A24" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="7">
+      <c r="B24" s="5"/>
+      <c r="C24" s="6">
         <v>1.5</v>
       </c>
-      <c r="D24" s="7">
+      <c r="D24" s="6">
         <v>1.5</v>
       </c>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1704,7 +1652,7 @@
         <f>IF('Raw Data'!K1="","",'Raw Data'!K1)</f>
         <v/>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="3" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1815,10 +1763,10 @@
         <f>IF('Raw Data'!O3="","",'Raw Data'!O3)</f>
         <v>Dp. Below sump I</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="Q3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="R3" s="4" t="s">
+      <c r="R3" s="3" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1854,8 +1802,8 @@
         <f>IF('Raw Data'!H4="","",'Raw Data'!H4)</f>
         <v>103</v>
       </c>
-      <c r="I4">
-        <f>IF('Raw Data'!I4="","",'Raw Data'!I4)</f>
+      <c r="I4" t="str">
+        <f>IF('Raw Data'!I4="","",SUBSTITUTE('Raw Data'!I4," ",":",1))</f>
         <v>283</v>
       </c>
       <c r="J4">
@@ -1882,12 +1830,12 @@
         <f>IF('Raw Data'!O4="","",'Raw Data'!O4)</f>
         <v/>
       </c>
-      <c r="Q4" s="5">
-        <f t="shared" ref="Q4:Q6" si="0">J4*COS(K4*PI()/180)</f>
+      <c r="Q4" s="4">
+        <f t="shared" ref="Q4" si="0">J4*COS(K4*PI()/180)</f>
         <v>20.769333130600252</v>
       </c>
-      <c r="R4" s="5">
-        <f t="shared" ref="R4:R6" si="1">J4*SIN(K4*PI()/180)</f>
+      <c r="R4" s="4">
+        <f t="shared" ref="R4" si="1">J4*SIN(K4*PI()/180)</f>
         <v>3.1039976337218231</v>
       </c>
     </row>
@@ -1923,8 +1871,9 @@
         <f>IF('Raw Data'!H5="","",'Raw Data'!H5)</f>
         <v>-</v>
       </c>
-      <c r="I5">
-        <v>322</v>
+      <c r="I5" t="str">
+        <f>IF('Raw Data'!I5="","",SUBSTITUTE('Raw Data'!I5," ",":",1))</f>
+        <v>322:30</v>
       </c>
       <c r="J5">
         <f>IF('Raw Data'!J5="","",'Raw Data'!J5)</f>
@@ -1950,12 +1899,12 @@
         <f>IF('Raw Data'!O5="","",'Raw Data'!O5)</f>
         <v>3.1</v>
       </c>
-      <c r="Q5" s="5">
-        <f t="shared" ref="Q5:Q35" si="2">J5*COS(K5*PI()/180)</f>
+      <c r="Q5" s="4">
+        <f t="shared" ref="Q5:Q23" si="2">J5*COS(K5*PI()/180)</f>
         <v>26.629711241505248</v>
       </c>
-      <c r="R5" s="5">
-        <f t="shared" ref="R5:R35" si="3">J5*SIN(K5*PI()/180)</f>
+      <c r="R5" s="4">
+        <f t="shared" ref="R5:R23" si="3">J5*SIN(K5*PI()/180)</f>
         <v>-4.4562853582382962</v>
       </c>
     </row>
@@ -1991,15 +1940,15 @@
         <f>IF('Raw Data'!H6="","",'Raw Data'!H6)</f>
         <v>83</v>
       </c>
-      <c r="I6">
-        <f>IF('Raw Data'!I6="","",'Raw Data'!I6)</f>
+      <c r="I6" t="str">
+        <f>IF('Raw Data'!I6="","",SUBSTITUTE('Raw Data'!I6," ",":",1))</f>
         <v>263</v>
       </c>
       <c r="J6">
         <f>IF('Raw Data'!J6="","",'Raw Data'!J6)</f>
         <v>37</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="2">
         <f>ASIN(N6/J6)*180/PI()</f>
         <v>2.3234386110520671</v>
       </c>
@@ -2019,11 +1968,11 @@
         <f>IF('Raw Data'!O6="","",'Raw Data'!O6)</f>
         <v>-1.4</v>
       </c>
-      <c r="Q6" s="5">
+      <c r="Q6" s="4">
         <f t="shared" si="2"/>
         <v>36.96958209122738</v>
       </c>
-      <c r="R6" s="5">
+      <c r="R6" s="4">
         <f t="shared" si="3"/>
         <v>1.5</v>
       </c>
@@ -2060,8 +2009,9 @@
         <f>IF('Raw Data'!H7="","",'Raw Data'!H7)</f>
         <v>-</v>
       </c>
-      <c r="I7">
-        <v>192</v>
+      <c r="I7" t="str">
+        <f>IF('Raw Data'!I7="","",SUBSTITUTE('Raw Data'!I7," ",":",1))</f>
+        <v>192:30</v>
       </c>
       <c r="J7">
         <f>IF('Raw Data'!J7="","",'Raw Data'!J7)</f>
@@ -2087,11 +2037,11 @@
         <f>IF('Raw Data'!O7="","",'Raw Data'!O7)</f>
         <v>0.1</v>
       </c>
-      <c r="Q7" s="5">
+      <c r="Q7" s="4">
         <f t="shared" si="2"/>
         <v>16.154399163106874</v>
       </c>
-      <c r="R7" s="5">
+      <c r="R7" s="4">
         <f t="shared" si="3"/>
         <v>1.2146553745865085</v>
       </c>
@@ -2128,8 +2078,8 @@
         <f>IF('Raw Data'!H8="","",'Raw Data'!H8)</f>
         <v>78</v>
       </c>
-      <c r="I8">
-        <f>IF('Raw Data'!I8="","",'Raw Data'!I8)</f>
+      <c r="I8" t="str">
+        <f>IF('Raw Data'!I8="","",SUBSTITUTE('Raw Data'!I8," ",":",1))</f>
         <v>258</v>
       </c>
       <c r="J8">
@@ -2156,11 +2106,11 @@
         <f>IF('Raw Data'!O8="","",'Raw Data'!O8)</f>
         <v>1.4</v>
       </c>
-      <c r="Q8" s="5">
+      <c r="Q8" s="4">
         <f t="shared" si="2"/>
         <v>46.799060814675357</v>
       </c>
-      <c r="R8" s="5">
+      <c r="R8" s="4">
         <f t="shared" si="3"/>
         <v>-4.3414176099883939</v>
       </c>
@@ -2197,15 +2147,15 @@
         <f>IF('Raw Data'!H9="","",'Raw Data'!H9)</f>
         <v>-</v>
       </c>
-      <c r="I9">
-        <f>IF('Raw Data'!I9="","",'Raw Data'!I9)</f>
+      <c r="I9" t="str">
+        <f>IF('Raw Data'!I9="","",SUBSTITUTE('Raw Data'!I9," ",":",1))</f>
         <v>292</v>
       </c>
       <c r="J9">
         <f>IF('Raw Data'!J9="","",'Raw Data'!J9)</f>
         <v>48</v>
       </c>
-      <c r="K9" s="3">
+      <c r="K9" s="2">
         <f>ASIN(N9/J9)*180/PI()</f>
         <v>-2.9855060057465379</v>
       </c>
@@ -2225,11 +2175,11 @@
         <f>IF('Raw Data'!O9="","",'Raw Data'!O9)</f>
         <v>-3.1</v>
       </c>
-      <c r="Q9" s="5">
+      <c r="Q9" s="4">
         <f t="shared" si="2"/>
         <v>47.934851621758462</v>
       </c>
-      <c r="R9" s="5">
+      <c r="R9" s="4">
         <f t="shared" si="3"/>
         <v>-2.5</v>
       </c>
@@ -2266,8 +2216,8 @@
         <f>IF('Raw Data'!H10="","",'Raw Data'!H10)</f>
         <v>159</v>
       </c>
-      <c r="I10">
-        <f>IF('Raw Data'!I10="","",'Raw Data'!I10)</f>
+      <c r="I10" t="str">
+        <f>IF('Raw Data'!I10="","",SUBSTITUTE('Raw Data'!I10," ",":",1))</f>
         <v>339</v>
       </c>
       <c r="J10">
@@ -2293,11 +2243,11 @@
         <f>IF('Raw Data'!O10="","",'Raw Data'!O10)</f>
         <v>-5.6</v>
       </c>
-      <c r="Q10" s="5">
+      <c r="Q10" s="4">
         <f t="shared" si="2"/>
         <v>36</v>
       </c>
-      <c r="R10" s="5">
+      <c r="R10" s="4">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -2334,8 +2284,8 @@
         <f>IF('Raw Data'!H11="","",'Raw Data'!H11)</f>
         <v>-</v>
       </c>
-      <c r="I11">
-        <f>IF('Raw Data'!I11="","",'Raw Data'!I11)</f>
+      <c r="I11" t="str">
+        <f>IF('Raw Data'!I11="","",SUBSTITUTE('Raw Data'!I11," ",":",1))</f>
         <v>247</v>
       </c>
       <c r="J11">
@@ -2362,11 +2312,11 @@
         <f>IF('Raw Data'!O11="","",'Raw Data'!O11)</f>
         <v>-5.6</v>
       </c>
-      <c r="Q11" s="5">
+      <c r="Q11" s="4">
         <f t="shared" si="2"/>
         <v>30.975026248547824</v>
       </c>
-      <c r="R11" s="5">
+      <c r="R11" s="4">
         <f t="shared" si="3"/>
         <v>-1.2440855685093515</v>
       </c>
@@ -2403,8 +2353,8 @@
         <f>IF('Raw Data'!H12="","",'Raw Data'!H12)</f>
         <v>95</v>
       </c>
-      <c r="I12">
-        <f>IF('Raw Data'!I12="","",'Raw Data'!I12)</f>
+      <c r="I12" t="str">
+        <f>IF('Raw Data'!I12="","",SUBSTITUTE('Raw Data'!I12," ",":",1))</f>
         <v>275</v>
       </c>
       <c r="J12">
@@ -2431,11 +2381,11 @@
         <f>IF('Raw Data'!O12="","",'Raw Data'!O12)</f>
         <v>-6.9</v>
       </c>
-      <c r="Q12" s="5">
+      <c r="Q12" s="4">
         <f t="shared" si="2"/>
         <v>25.984161502496491</v>
       </c>
-      <c r="R12" s="5">
+      <c r="R12" s="4">
         <f t="shared" si="3"/>
         <v>0.90738691426502516</v>
       </c>
@@ -2472,8 +2422,8 @@
         <f>IF('Raw Data'!H13="","",'Raw Data'!H13)</f>
         <v>-</v>
       </c>
-      <c r="I13">
-        <f>IF('Raw Data'!I13="","",'Raw Data'!I13)</f>
+      <c r="I13" t="str">
+        <f>IF('Raw Data'!I13="","",SUBSTITUTE('Raw Data'!I13," ",":",1))</f>
         <v>320</v>
       </c>
       <c r="J13">
@@ -2500,11 +2450,11 @@
         <f>IF('Raw Data'!O13="","",'Raw Data'!O13)</f>
         <v>-6</v>
       </c>
-      <c r="Q13" s="5">
+      <c r="Q13" s="4">
         <f t="shared" si="2"/>
         <v>26.495963921644368</v>
       </c>
-      <c r="R13" s="5">
+      <c r="R13" s="4">
         <f t="shared" si="3"/>
         <v>0.46248877058801308</v>
       </c>
@@ -2541,8 +2491,8 @@
         <f>IF('Raw Data'!H14="","",'Raw Data'!H14)</f>
         <v>193</v>
       </c>
-      <c r="I14">
-        <f>IF('Raw Data'!I14="","",'Raw Data'!I14)</f>
+      <c r="I14" t="str">
+        <f>IF('Raw Data'!I14="","",SUBSTITUTE('Raw Data'!I14," ",":",1))</f>
         <v>13</v>
       </c>
       <c r="J14">
@@ -2569,11 +2519,11 @@
         <f>IF('Raw Data'!O14="","",'Raw Data'!O14)</f>
         <v>-5.5</v>
       </c>
-      <c r="Q14" s="5">
+      <c r="Q14" s="4">
         <f t="shared" si="2"/>
         <v>17.28454596041491</v>
       </c>
-      <c r="R14" s="5">
+      <c r="R14" s="4">
         <f t="shared" si="3"/>
         <v>-2.7376031382040402</v>
       </c>
@@ -2610,8 +2560,8 @@
         <f>IF('Raw Data'!H15="","",'Raw Data'!H15)</f>
         <v>-</v>
       </c>
-      <c r="I15">
-        <f>IF('Raw Data'!I15="","",'Raw Data'!I15)</f>
+      <c r="I15" t="str">
+        <f>IF('Raw Data'!I15="","",SUBSTITUTE('Raw Data'!I15," ",":",1))</f>
         <v>299</v>
       </c>
       <c r="J15">
@@ -2638,11 +2588,11 @@
         <f>IF('Raw Data'!O15="","",'Raw Data'!O15)</f>
         <v>-8.1999999999999993</v>
       </c>
-      <c r="Q15" s="5">
+      <c r="Q15" s="4">
         <f t="shared" si="2"/>
         <v>32.954774646900937</v>
       </c>
-      <c r="R15" s="5">
+      <c r="R15" s="4">
         <f t="shared" si="3"/>
         <v>-1.7270865560171462</v>
       </c>
@@ -2679,8 +2629,8 @@
         <f>IF('Raw Data'!H16="","",'Raw Data'!H16)</f>
         <v>142</v>
       </c>
-      <c r="I16">
-        <f>IF('Raw Data'!I16="","",'Raw Data'!I16)</f>
+      <c r="I16" t="str">
+        <f>IF('Raw Data'!I16="","",SUBSTITUTE('Raw Data'!I16," ",":",1))</f>
         <v>322</v>
       </c>
       <c r="J16">
@@ -2707,11 +2657,11 @@
         <f>IF('Raw Data'!O16="","",'Raw Data'!O16)</f>
         <v>-9.9</v>
       </c>
-      <c r="Q16" s="5">
+      <c r="Q16" s="4">
         <f t="shared" si="2"/>
         <v>42.651461031371277</v>
       </c>
-      <c r="R16" s="5">
+      <c r="R16" s="4">
         <f t="shared" si="3"/>
         <v>-5.4637781698580703</v>
       </c>
@@ -2748,8 +2698,8 @@
         <f>IF('Raw Data'!H17="","",'Raw Data'!H17)</f>
         <v>-</v>
       </c>
-      <c r="I17">
-        <f>IF('Raw Data'!I17="","",'Raw Data'!I17)</f>
+      <c r="I17" t="str">
+        <f>IF('Raw Data'!I17="","",SUBSTITUTE('Raw Data'!I17," ",":",1))</f>
         <v>281</v>
       </c>
       <c r="J17">
@@ -2776,11 +2726,11 @@
         <f>IF('Raw Data'!O17="","",'Raw Data'!O17)</f>
         <v>-15.5</v>
       </c>
-      <c r="Q17" s="5">
+      <c r="Q17" s="4">
         <f t="shared" si="2"/>
         <v>15.490557818795985</v>
       </c>
-      <c r="R17" s="5">
+      <c r="R17" s="4">
         <f t="shared" si="3"/>
         <v>-0.54094219888876505</v>
       </c>
@@ -2817,8 +2767,8 @@
         <f>IF('Raw Data'!H18="","",'Raw Data'!H18)</f>
         <v>127</v>
       </c>
-      <c r="I18">
-        <f>IF('Raw Data'!I18="","",'Raw Data'!I18)</f>
+      <c r="I18" t="str">
+        <f>IF('Raw Data'!I18="","",SUBSTITUTE('Raw Data'!I18," ",":",1))</f>
         <v>307</v>
       </c>
       <c r="J18">
@@ -2845,11 +2795,11 @@
         <f>IF('Raw Data'!O18="","",'Raw Data'!O18)</f>
         <v>-16</v>
       </c>
-      <c r="Q18" s="5">
+      <c r="Q18" s="4">
         <f t="shared" si="2"/>
         <v>55.786903093137752</v>
       </c>
-      <c r="R18" s="5">
+      <c r="R18" s="4">
         <f t="shared" si="3"/>
         <v>-4.8807215938688575</v>
       </c>
@@ -2886,8 +2836,8 @@
         <f>IF('Raw Data'!H19="","",'Raw Data'!H19)</f>
         <v>-</v>
       </c>
-      <c r="I19">
-        <f>IF('Raw Data'!I19="","",'Raw Data'!I19)</f>
+      <c r="I19" t="str">
+        <f>IF('Raw Data'!I19="","",SUBSTITUTE('Raw Data'!I19," ",":",1))</f>
         <v>283</v>
       </c>
       <c r="J19">
@@ -2914,11 +2864,11 @@
         <f>IF('Raw Data'!O19="","",'Raw Data'!O19)</f>
         <v>-20.9</v>
       </c>
-      <c r="Q19" s="5">
+      <c r="Q19" s="4">
         <f t="shared" si="2"/>
         <v>15.799945854284561</v>
       </c>
-      <c r="R19" s="5">
+      <c r="R19" s="4">
         <f t="shared" si="3"/>
         <v>-4.1364256021204297E-2</v>
       </c>
@@ -2955,15 +2905,15 @@
         <f>IF('Raw Data'!H20="","",'Raw Data'!H20)</f>
         <v>37</v>
       </c>
-      <c r="I20">
-        <f>IF('Raw Data'!I20="","",'Raw Data'!I20)</f>
+      <c r="I20" t="str">
+        <f>IF('Raw Data'!I20="","",SUBSTITUTE('Raw Data'!I20," ",":",1))</f>
         <v>217</v>
       </c>
       <c r="J20">
         <f>IF('Raw Data'!J20="","",'Raw Data'!J20)</f>
         <v>15.3</v>
       </c>
-      <c r="K20" s="3">
+      <c r="K20" s="2">
         <f>ASIN(N20/J20)*180/PI()</f>
         <v>-15.155399662290439</v>
       </c>
@@ -2983,11 +2933,11 @@
         <f>IF('Raw Data'!O20="","",'Raw Data'!O20)</f>
         <v>-21</v>
       </c>
-      <c r="Q20" s="5">
+      <c r="Q20" s="4">
         <f t="shared" si="2"/>
         <v>14.767870530310049</v>
       </c>
-      <c r="R20" s="5">
+      <c r="R20" s="4">
         <f t="shared" si="3"/>
         <v>-4</v>
       </c>
@@ -3024,15 +2974,15 @@
         <f>IF('Raw Data'!H21="","",'Raw Data'!H21)</f>
         <v>-</v>
       </c>
-      <c r="I21">
-        <f>IF('Raw Data'!I21="","",'Raw Data'!I21)</f>
+      <c r="I21" t="str">
+        <f>IF('Raw Data'!I21="","",SUBSTITUTE('Raw Data'!I21," ",":",1))</f>
         <v>310</v>
       </c>
       <c r="J21">
         <f>IF('Raw Data'!J21="","",'Raw Data'!J21)</f>
         <v>39.5</v>
       </c>
-      <c r="K21" s="3">
+      <c r="K21" s="2">
         <f>ASIN(N21/J21)*180/PI()</f>
         <v>5.8120668348260685</v>
       </c>
@@ -3052,11 +3002,11 @@
         <f>IF('Raw Data'!O21="","",'Raw Data'!O21)</f>
         <v>-25</v>
       </c>
-      <c r="Q21" s="5">
+      <c r="Q21" s="4">
         <f t="shared" si="2"/>
         <v>39.296946446257117</v>
       </c>
-      <c r="R21" s="5">
+      <c r="R21" s="4">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
@@ -3093,8 +3043,8 @@
         <f>IF('Raw Data'!H22="","",'Raw Data'!H22)</f>
         <v>58</v>
       </c>
-      <c r="I22">
-        <f>IF('Raw Data'!I22="","",'Raw Data'!I22)</f>
+      <c r="I22" t="str">
+        <f>IF('Raw Data'!I22="","",SUBSTITUTE('Raw Data'!I22," ",":",1))</f>
         <v>238</v>
       </c>
       <c r="J22">
@@ -3121,11 +3071,11 @@
         <f>IF('Raw Data'!O22="","",'Raw Data'!O22)</f>
         <v>-21</v>
       </c>
-      <c r="Q22" s="5">
+      <c r="Q22" s="4">
         <f t="shared" si="2"/>
         <v>39.556039048494014</v>
       </c>
-      <c r="R22" s="5">
+      <c r="R22" s="4">
         <f t="shared" si="3"/>
         <v>-1.8654154481018492</v>
       </c>
@@ -3162,15 +3112,15 @@
         <f>IF('Raw Data'!H23="","",'Raw Data'!H23)</f>
         <v>-</v>
       </c>
-      <c r="I23">
-        <f>IF('Raw Data'!I23="","",'Raw Data'!I23)</f>
+      <c r="I23" t="str">
+        <f>IF('Raw Data'!I23="","",SUBSTITUTE('Raw Data'!I23," ",":",1))</f>
         <v>148</v>
       </c>
       <c r="J23">
         <f>IF('Raw Data'!J23="","",'Raw Data'!J23)</f>
         <v>49</v>
       </c>
-      <c r="K23" s="3">
+      <c r="K23" s="2">
         <f>ASIN(N23/J23)*180/PI()</f>
         <v>-1.9882117515894562</v>
       </c>
@@ -3190,11 +3140,11 @@
         <f>IF('Raw Data'!O23="","",'Raw Data'!O23)</f>
         <v>-22.9</v>
       </c>
-      <c r="Q23" s="5">
+      <c r="Q23" s="4">
         <f t="shared" si="2"/>
         <v>48.970501324777146</v>
       </c>
-      <c r="R23" s="5">
+      <c r="R23" s="4">
         <f t="shared" si="3"/>
         <v>-1.7</v>
       </c>
@@ -3259,61 +3209,61 @@
         <f>IF('Raw Data'!O24="","",'Raw Data'!O24)</f>
         <v/>
       </c>
-      <c r="Q24" s="5"/>
-      <c r="R24" s="5"/>
+      <c r="Q24" s="4"/>
+      <c r="R24" s="4"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="Q25" s="5"/>
-      <c r="R25" s="5"/>
+      <c r="Q25" s="4"/>
+      <c r="R25" s="4"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="Q26" s="5"/>
-      <c r="R26" s="5"/>
+      <c r="Q26" s="4"/>
+      <c r="R26" s="4"/>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="Q27" s="5"/>
-      <c r="R27" s="5"/>
+      <c r="Q27" s="4"/>
+      <c r="R27" s="4"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="Q28" s="5"/>
-      <c r="R28" s="5"/>
+      <c r="Q28" s="4"/>
+      <c r="R28" s="4"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="Q29" s="5"/>
-      <c r="R29" s="5"/>
+      <c r="Q29" s="4"/>
+      <c r="R29" s="4"/>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="Q30" s="5"/>
-      <c r="R30" s="5"/>
+      <c r="Q30" s="4"/>
+      <c r="R30" s="4"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="Q31" s="5"/>
-      <c r="R31" s="5"/>
+      <c r="Q31" s="4"/>
+      <c r="R31" s="4"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="Q32" s="5"/>
-      <c r="R32" s="5"/>
+      <c r="Q32" s="4"/>
+      <c r="R32" s="4"/>
     </row>
     <row r="33" spans="17:18" x14ac:dyDescent="0.25">
-      <c r="Q33" s="5"/>
-      <c r="R33" s="5"/>
+      <c r="Q33" s="4"/>
+      <c r="R33" s="4"/>
     </row>
     <row r="34" spans="17:18" x14ac:dyDescent="0.25">
-      <c r="Q34" s="5"/>
-      <c r="R34" s="5"/>
+      <c r="Q34" s="4"/>
+      <c r="R34" s="4"/>
     </row>
     <row r="35" spans="17:18" x14ac:dyDescent="0.25">
-      <c r="Q35" s="5"/>
-      <c r="R35" s="5"/>
+      <c r="Q35" s="4"/>
+      <c r="R35" s="4"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="Q24:Q35 Q4:R23">
-    <cfRule type="expression" dxfId="8" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>Q4-M4&gt;0.15</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R24:R35">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>R24-N24&gt;0.1</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3353,15 +3303,15 @@
         <f>'Interpreted Data'!B4</f>
         <v>B</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <f>'Interpreted Data'!J4/'Interpreted Data'!$H$1</f>
         <v>6.4024390243902447</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="9" t="str">
         <f>'Interpreted Data'!I4</f>
         <v>283</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="10">
         <f>'Interpreted Data'!K4</f>
         <v>8.5</v>
       </c>
@@ -3375,15 +3325,15 @@
         <f>'Interpreted Data'!B5</f>
         <v>C</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <f>'Interpreted Data'!J5/'Interpreted Data'!$H$1</f>
         <v>8.2317073170731714</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="9" t="str">
         <f>'Interpreted Data'!I5</f>
-        <v>322</v>
-      </c>
-      <c r="E5">
+        <v>322:30</v>
+      </c>
+      <c r="E5" s="10">
         <f>'Interpreted Data'!K5</f>
         <v>-9.5</v>
       </c>
@@ -3397,15 +3347,15 @@
         <f>'Interpreted Data'!B6</f>
         <v>D</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <f>'Interpreted Data'!J6/'Interpreted Data'!$H$1</f>
         <v>11.280487804878049</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="9" t="str">
         <f>'Interpreted Data'!I6</f>
         <v>263</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="10">
         <f>'Interpreted Data'!K6</f>
         <v>2.3234386110520671</v>
       </c>
@@ -3419,15 +3369,15 @@
         <f>'Interpreted Data'!B7</f>
         <v>E</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <f>'Interpreted Data'!J7/'Interpreted Data'!$H$1</f>
         <v>4.9390243902439028</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="9" t="str">
         <f>'Interpreted Data'!I7</f>
-        <v>192</v>
-      </c>
-      <c r="E7">
+        <v>192:30</v>
+      </c>
+      <c r="E7" s="10">
         <f>'Interpreted Data'!K7</f>
         <v>4.3</v>
       </c>
@@ -3441,15 +3391,15 @@
         <f>'Interpreted Data'!B8</f>
         <v>F</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <f>'Interpreted Data'!J8/'Interpreted Data'!$H$1</f>
         <v>14.329268292682928</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="9" t="str">
         <f>'Interpreted Data'!I8</f>
         <v>258</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="10">
         <f>'Interpreted Data'!K8</f>
         <v>-5.3</v>
       </c>
@@ -3463,15 +3413,15 @@
         <f>'Interpreted Data'!B9</f>
         <v>G</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <f>'Interpreted Data'!J9/'Interpreted Data'!$H$1</f>
         <v>14.634146341463415</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="9" t="str">
         <f>'Interpreted Data'!I9</f>
         <v>292</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="10">
         <f>'Interpreted Data'!K9</f>
         <v>-2.9855060057465379</v>
       </c>
@@ -3485,15 +3435,15 @@
         <f>'Interpreted Data'!B10</f>
         <v>H</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <f>'Interpreted Data'!J10/'Interpreted Data'!$H$1</f>
         <v>10.975609756097562</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="9" t="str">
         <f>'Interpreted Data'!I10</f>
         <v>339</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="10">
         <f>'Interpreted Data'!K10</f>
         <v>0</v>
       </c>
@@ -3507,15 +3457,15 @@
         <f>'Interpreted Data'!B11</f>
         <v>I</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <f>'Interpreted Data'!J11/'Interpreted Data'!$H$1</f>
         <v>9.4512195121951219</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="9" t="str">
         <f>'Interpreted Data'!I11</f>
         <v>247</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="10">
         <f>'Interpreted Data'!K11</f>
         <v>-2.2999999999999998</v>
       </c>
@@ -3529,15 +3479,15 @@
         <f>'Interpreted Data'!B12</f>
         <v>J</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="2">
         <f>'Interpreted Data'!J12/'Interpreted Data'!$H$1</f>
         <v>7.9268292682926838</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="9" t="str">
         <f>'Interpreted Data'!I12</f>
         <v>275</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="10">
         <f>'Interpreted Data'!K12</f>
         <v>2</v>
       </c>
@@ -3551,15 +3501,15 @@
         <f>'Interpreted Data'!B13</f>
         <v>K</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="2">
         <f>'Interpreted Data'!J13/'Interpreted Data'!$H$1</f>
         <v>8.0792682926829276</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="9" t="str">
         <f>'Interpreted Data'!I13</f>
         <v>320</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="10">
         <f>'Interpreted Data'!K13</f>
         <v>1</v>
       </c>
@@ -3573,15 +3523,15 @@
         <f>'Interpreted Data'!B14</f>
         <v>L</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="2">
         <f>'Interpreted Data'!J14/'Interpreted Data'!$H$1</f>
         <v>5.3353658536585371</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="9" t="str">
         <f>'Interpreted Data'!I14</f>
         <v>13</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="10">
         <f>'Interpreted Data'!K14</f>
         <v>-9</v>
       </c>
@@ -3595,15 +3545,15 @@
         <f>'Interpreted Data'!B15</f>
         <v>M</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="2">
         <f>'Interpreted Data'!J15/'Interpreted Data'!$H$1</f>
         <v>10.060975609756099</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="9" t="str">
         <f>'Interpreted Data'!I15</f>
         <v>299</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="10">
         <f>'Interpreted Data'!K15</f>
         <v>-3</v>
       </c>
@@ -3617,15 +3567,15 @@
         <f>'Interpreted Data'!B16</f>
         <v>N</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="2">
         <f>'Interpreted Data'!J16/'Interpreted Data'!$H$1</f>
         <v>13.109756097560977</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="9" t="str">
         <f>'Interpreted Data'!I16</f>
         <v>322</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="10">
         <f>'Interpreted Data'!K16</f>
         <v>-7.3</v>
       </c>
@@ -3639,15 +3589,15 @@
         <f>'Interpreted Data'!B17</f>
         <v>O</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="2">
         <f>'Interpreted Data'!J17/'Interpreted Data'!$H$1</f>
         <v>4.725609756097561</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="9" t="str">
         <f>'Interpreted Data'!I17</f>
         <v>281</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="10">
         <f>'Interpreted Data'!K17</f>
         <v>-2</v>
       </c>
@@ -3661,15 +3611,15 @@
         <f>'Interpreted Data'!B18</f>
         <v>P</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="2">
         <f>'Interpreted Data'!J18/'Interpreted Data'!$H$1</f>
         <v>17.073170731707318</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="9" t="str">
         <f>'Interpreted Data'!I18</f>
         <v>307</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="10">
         <f>'Interpreted Data'!K18</f>
         <v>-5</v>
       </c>
@@ -3683,15 +3633,15 @@
         <f>'Interpreted Data'!B19</f>
         <v>Q</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="2">
         <f>'Interpreted Data'!J19/'Interpreted Data'!$H$1</f>
         <v>4.8170731707317076</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="9" t="str">
         <f>'Interpreted Data'!I19</f>
         <v>283</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="10">
         <f>'Interpreted Data'!K19</f>
         <v>-0.15</v>
       </c>
@@ -3705,15 +3655,15 @@
         <f>'Interpreted Data'!B20</f>
         <v>R</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="2">
         <f>'Interpreted Data'!J20/'Interpreted Data'!$H$1</f>
         <v>4.6646341463414638</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="9" t="str">
         <f>'Interpreted Data'!I20</f>
         <v>217</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="10">
         <f>'Interpreted Data'!K20</f>
         <v>-15.155399662290439</v>
       </c>
@@ -3727,15 +3677,15 @@
         <f>'Interpreted Data'!B21</f>
         <v>S</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="2">
         <f>'Interpreted Data'!J21/'Interpreted Data'!$H$1</f>
         <v>12.042682926829269</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="9" t="str">
         <f>'Interpreted Data'!I21</f>
         <v>310</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="10">
         <f>'Interpreted Data'!K21</f>
         <v>5.8120668348260685</v>
       </c>
@@ -3749,15 +3699,15 @@
         <f>'Interpreted Data'!B22</f>
         <v>T</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C22" s="2">
         <f>'Interpreted Data'!J22/'Interpreted Data'!$H$1</f>
         <v>12.073170731707318</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="9" t="str">
         <f>'Interpreted Data'!I22</f>
         <v>238</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="10">
         <f>'Interpreted Data'!K22</f>
         <v>-2.7</v>
       </c>
@@ -3771,24 +3721,501 @@
         <f>'Interpreted Data'!B23</f>
         <v>U</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C23" s="2">
         <f>'Interpreted Data'!J23/'Interpreted Data'!$H$1</f>
         <v>14.939024390243903</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="9" t="str">
         <f>'Interpreted Data'!I23</f>
         <v>148</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="10">
         <f>'Interpreted Data'!K23</f>
         <v>-1.9882117515894562</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C24" s="3"/>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C25" s="3"/>
+      <c r="C25" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A4:E25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f>'Interpreted Data'!A4</f>
+        <v>A</v>
+      </c>
+      <c r="B4" t="str">
+        <f>'Interpreted Data'!B4</f>
+        <v>B</v>
+      </c>
+      <c r="C4" s="2">
+        <f>'Interpreted Data'!J4</f>
+        <v>21</v>
+      </c>
+      <c r="D4" s="9" t="str">
+        <f>'Interpreted Data'!I4</f>
+        <v>283</v>
+      </c>
+      <c r="E4" s="10">
+        <f>'Interpreted Data'!K4</f>
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <f>'Interpreted Data'!A5</f>
+        <v>B</v>
+      </c>
+      <c r="B5" t="str">
+        <f>'Interpreted Data'!B5</f>
+        <v>C</v>
+      </c>
+      <c r="C5" s="2">
+        <f>'Interpreted Data'!J5</f>
+        <v>27</v>
+      </c>
+      <c r="D5" s="9" t="str">
+        <f>'Interpreted Data'!I5</f>
+        <v>322:30</v>
+      </c>
+      <c r="E5" s="10">
+        <f>'Interpreted Data'!K5</f>
+        <v>-9.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <f>'Interpreted Data'!A6</f>
+        <v>C</v>
+      </c>
+      <c r="B6" t="str">
+        <f>'Interpreted Data'!B6</f>
+        <v>D</v>
+      </c>
+      <c r="C6" s="2">
+        <f>'Interpreted Data'!J6</f>
+        <v>37</v>
+      </c>
+      <c r="D6" s="9" t="str">
+        <f>'Interpreted Data'!I6</f>
+        <v>263</v>
+      </c>
+      <c r="E6" s="10">
+        <f>'Interpreted Data'!K6</f>
+        <v>2.3234386110520671</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <f>'Interpreted Data'!A7</f>
+        <v>D</v>
+      </c>
+      <c r="B7" t="str">
+        <f>'Interpreted Data'!B7</f>
+        <v>E</v>
+      </c>
+      <c r="C7" s="2">
+        <f>'Interpreted Data'!J7</f>
+        <v>16.2</v>
+      </c>
+      <c r="D7" s="9" t="str">
+        <f>'Interpreted Data'!I7</f>
+        <v>192:30</v>
+      </c>
+      <c r="E7" s="10">
+        <f>'Interpreted Data'!K7</f>
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <f>'Interpreted Data'!A8</f>
+        <v>E</v>
+      </c>
+      <c r="B8" t="str">
+        <f>'Interpreted Data'!B8</f>
+        <v>F</v>
+      </c>
+      <c r="C8" s="2">
+        <f>'Interpreted Data'!J8</f>
+        <v>47</v>
+      </c>
+      <c r="D8" s="9" t="str">
+        <f>'Interpreted Data'!I8</f>
+        <v>258</v>
+      </c>
+      <c r="E8" s="10">
+        <f>'Interpreted Data'!K8</f>
+        <v>-5.3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <f>'Interpreted Data'!A9</f>
+        <v>F</v>
+      </c>
+      <c r="B9" t="str">
+        <f>'Interpreted Data'!B9</f>
+        <v>G</v>
+      </c>
+      <c r="C9" s="2">
+        <f>'Interpreted Data'!J9</f>
+        <v>48</v>
+      </c>
+      <c r="D9" s="9" t="str">
+        <f>'Interpreted Data'!I9</f>
+        <v>292</v>
+      </c>
+      <c r="E9" s="10">
+        <f>'Interpreted Data'!K9</f>
+        <v>-2.9855060057465379</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="str">
+        <f>'Interpreted Data'!A10</f>
+        <v>G</v>
+      </c>
+      <c r="B10" t="str">
+        <f>'Interpreted Data'!B10</f>
+        <v>H</v>
+      </c>
+      <c r="C10" s="2">
+        <f>'Interpreted Data'!J10</f>
+        <v>36</v>
+      </c>
+      <c r="D10" s="9" t="str">
+        <f>'Interpreted Data'!I10</f>
+        <v>339</v>
+      </c>
+      <c r="E10" s="10">
+        <f>'Interpreted Data'!K10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="str">
+        <f>'Interpreted Data'!A11</f>
+        <v>H</v>
+      </c>
+      <c r="B11" t="str">
+        <f>'Interpreted Data'!B11</f>
+        <v>I</v>
+      </c>
+      <c r="C11" s="2">
+        <f>'Interpreted Data'!J11</f>
+        <v>31</v>
+      </c>
+      <c r="D11" s="9" t="str">
+        <f>'Interpreted Data'!I11</f>
+        <v>247</v>
+      </c>
+      <c r="E11" s="10">
+        <f>'Interpreted Data'!K11</f>
+        <v>-2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="str">
+        <f>'Interpreted Data'!A12</f>
+        <v>I</v>
+      </c>
+      <c r="B12" t="str">
+        <f>'Interpreted Data'!B12</f>
+        <v>J</v>
+      </c>
+      <c r="C12" s="2">
+        <f>'Interpreted Data'!J12</f>
+        <v>26</v>
+      </c>
+      <c r="D12" s="9" t="str">
+        <f>'Interpreted Data'!I12</f>
+        <v>275</v>
+      </c>
+      <c r="E12" s="10">
+        <f>'Interpreted Data'!K12</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="str">
+        <f>'Interpreted Data'!A13</f>
+        <v>J</v>
+      </c>
+      <c r="B13" t="str">
+        <f>'Interpreted Data'!B13</f>
+        <v>K</v>
+      </c>
+      <c r="C13" s="2">
+        <f>'Interpreted Data'!J13</f>
+        <v>26.5</v>
+      </c>
+      <c r="D13" s="9" t="str">
+        <f>'Interpreted Data'!I13</f>
+        <v>320</v>
+      </c>
+      <c r="E13" s="10">
+        <f>'Interpreted Data'!K13</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="str">
+        <f>'Interpreted Data'!A14</f>
+        <v>K</v>
+      </c>
+      <c r="B14" t="str">
+        <f>'Interpreted Data'!B14</f>
+        <v>L</v>
+      </c>
+      <c r="C14" s="2">
+        <f>'Interpreted Data'!J14</f>
+        <v>17.5</v>
+      </c>
+      <c r="D14" s="9" t="str">
+        <f>'Interpreted Data'!I14</f>
+        <v>13</v>
+      </c>
+      <c r="E14" s="10">
+        <f>'Interpreted Data'!K14</f>
+        <v>-9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="str">
+        <f>'Interpreted Data'!A15</f>
+        <v>L</v>
+      </c>
+      <c r="B15" t="str">
+        <f>'Interpreted Data'!B15</f>
+        <v>M</v>
+      </c>
+      <c r="C15" s="2">
+        <f>'Interpreted Data'!J15</f>
+        <v>33</v>
+      </c>
+      <c r="D15" s="9" t="str">
+        <f>'Interpreted Data'!I15</f>
+        <v>299</v>
+      </c>
+      <c r="E15" s="10">
+        <f>'Interpreted Data'!K15</f>
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="str">
+        <f>'Interpreted Data'!A16</f>
+        <v>M</v>
+      </c>
+      <c r="B16" t="str">
+        <f>'Interpreted Data'!B16</f>
+        <v>N</v>
+      </c>
+      <c r="C16" s="2">
+        <f>'Interpreted Data'!J16</f>
+        <v>43</v>
+      </c>
+      <c r="D16" s="9" t="str">
+        <f>'Interpreted Data'!I16</f>
+        <v>322</v>
+      </c>
+      <c r="E16" s="10">
+        <f>'Interpreted Data'!K16</f>
+        <v>-7.3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="str">
+        <f>'Interpreted Data'!A17</f>
+        <v>N</v>
+      </c>
+      <c r="B17" t="str">
+        <f>'Interpreted Data'!B17</f>
+        <v>O</v>
+      </c>
+      <c r="C17" s="2">
+        <f>'Interpreted Data'!J17</f>
+        <v>15.5</v>
+      </c>
+      <c r="D17" s="9" t="str">
+        <f>'Interpreted Data'!I17</f>
+        <v>281</v>
+      </c>
+      <c r="E17" s="10">
+        <f>'Interpreted Data'!K17</f>
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="str">
+        <f>'Interpreted Data'!A18</f>
+        <v>O</v>
+      </c>
+      <c r="B18" t="str">
+        <f>'Interpreted Data'!B18</f>
+        <v>P</v>
+      </c>
+      <c r="C18" s="2">
+        <f>'Interpreted Data'!J18</f>
+        <v>56</v>
+      </c>
+      <c r="D18" s="9" t="str">
+        <f>'Interpreted Data'!I18</f>
+        <v>307</v>
+      </c>
+      <c r="E18" s="10">
+        <f>'Interpreted Data'!K18</f>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="str">
+        <f>'Interpreted Data'!A19</f>
+        <v>P</v>
+      </c>
+      <c r="B19" t="str">
+        <f>'Interpreted Data'!B19</f>
+        <v>Q</v>
+      </c>
+      <c r="C19" s="2">
+        <f>'Interpreted Data'!J19</f>
+        <v>15.8</v>
+      </c>
+      <c r="D19" s="9" t="str">
+        <f>'Interpreted Data'!I19</f>
+        <v>283</v>
+      </c>
+      <c r="E19" s="10">
+        <f>'Interpreted Data'!K19</f>
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="str">
+        <f>'Interpreted Data'!A20</f>
+        <v>Q</v>
+      </c>
+      <c r="B20" t="str">
+        <f>'Interpreted Data'!B20</f>
+        <v>R</v>
+      </c>
+      <c r="C20" s="2">
+        <f>'Interpreted Data'!J20</f>
+        <v>15.3</v>
+      </c>
+      <c r="D20" s="9" t="str">
+        <f>'Interpreted Data'!I20</f>
+        <v>217</v>
+      </c>
+      <c r="E20" s="10">
+        <f>'Interpreted Data'!K20</f>
+        <v>-15.155399662290439</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="str">
+        <f>'Interpreted Data'!A21</f>
+        <v>R</v>
+      </c>
+      <c r="B21" t="str">
+        <f>'Interpreted Data'!B21</f>
+        <v>S</v>
+      </c>
+      <c r="C21" s="2">
+        <f>'Interpreted Data'!J21</f>
+        <v>39.5</v>
+      </c>
+      <c r="D21" s="9" t="str">
+        <f>'Interpreted Data'!I21</f>
+        <v>310</v>
+      </c>
+      <c r="E21" s="10">
+        <f>'Interpreted Data'!K21</f>
+        <v>5.8120668348260685</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="str">
+        <f>'Interpreted Data'!A22</f>
+        <v>S</v>
+      </c>
+      <c r="B22" t="str">
+        <f>'Interpreted Data'!B22</f>
+        <v>T</v>
+      </c>
+      <c r="C22" s="2">
+        <f>'Interpreted Data'!J22</f>
+        <v>39.6</v>
+      </c>
+      <c r="D22" s="9" t="str">
+        <f>'Interpreted Data'!I22</f>
+        <v>238</v>
+      </c>
+      <c r="E22" s="10">
+        <f>'Interpreted Data'!K22</f>
+        <v>-2.7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="str">
+        <f>'Interpreted Data'!A23</f>
+        <v>T</v>
+      </c>
+      <c r="B23" t="str">
+        <f>'Interpreted Data'!B23</f>
+        <v>U</v>
+      </c>
+      <c r="C23" s="2">
+        <f>'Interpreted Data'!J23</f>
+        <v>49</v>
+      </c>
+      <c r="D23" s="9" t="str">
+        <f>'Interpreted Data'!I23</f>
+        <v>148</v>
+      </c>
+      <c r="E23" s="10">
+        <f>'Interpreted Data'!K23</f>
+        <v>-1.9882117515894562</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="str">
+        <f>'Interpreted Data'!A24</f>
+        <v>U</v>
+      </c>
+      <c r="B24" t="str">
+        <f>'Interpreted Data'!B24</f>
+        <v/>
+      </c>
+      <c r="C24" s="2" t="str">
+        <f>'Interpreted Data'!J24</f>
+        <v/>
+      </c>
+      <c r="D24" s="9" t="str">
+        <f>'Interpreted Data'!I24</f>
+        <v/>
+      </c>
+      <c r="E24" s="10" t="str">
+        <f>'Interpreted Data'!K24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C25" s="2"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>